<commit_message>
daily auto push: 2026-03-12 04:20 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3280"/>
+  <dimension ref="A1:D3281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58719,12 +58719,12 @@
     <row r="3239">
       <c r="A3239" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/03/12</t>
         </is>
       </c>
       <c r="B3239" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3239" t="n">
@@ -58746,7 +58746,7 @@
         </is>
       </c>
       <c r="C3240" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3240" t="n">
         <v>3</v>
@@ -58764,7 +58764,7 @@
         </is>
       </c>
       <c r="C3241" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3241" t="n">
         <v>3</v>
@@ -58782,7 +58782,7 @@
         </is>
       </c>
       <c r="C3242" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3242" t="n">
         <v>3</v>
@@ -58791,16 +58791,16 @@
     <row r="3243">
       <c r="A3243" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3243" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3243" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3243" t="n">
         <v>3</v>
@@ -58818,7 +58818,7 @@
         </is>
       </c>
       <c r="C3244" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3244" t="n">
         <v>3</v>
@@ -58836,7 +58836,7 @@
         </is>
       </c>
       <c r="C3245" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3245" t="n">
         <v>3</v>
@@ -58854,7 +58854,7 @@
         </is>
       </c>
       <c r="C3246" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3246" t="n">
         <v>3</v>
@@ -58872,7 +58872,7 @@
         </is>
       </c>
       <c r="C3247" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3247" t="n">
         <v>3</v>
@@ -58890,7 +58890,7 @@
         </is>
       </c>
       <c r="C3248" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3248" t="n">
         <v>3</v>
@@ -58899,16 +58899,16 @@
     <row r="3249">
       <c r="A3249" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3249" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3249" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3249" t="n">
         <v>3</v>
@@ -58926,7 +58926,7 @@
         </is>
       </c>
       <c r="C3250" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3250" t="n">
         <v>3</v>
@@ -58944,7 +58944,7 @@
         </is>
       </c>
       <c r="C3251" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3251" t="n">
         <v>3</v>
@@ -58962,7 +58962,7 @@
         </is>
       </c>
       <c r="C3252" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3252" t="n">
         <v>3</v>
@@ -58980,7 +58980,7 @@
         </is>
       </c>
       <c r="C3253" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3253" t="n">
         <v>3</v>
@@ -58998,7 +58998,7 @@
         </is>
       </c>
       <c r="C3254" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3254" t="n">
         <v>3</v>
@@ -59007,16 +59007,16 @@
     <row r="3255">
       <c r="A3255" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3255" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3255" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3255" t="n">
         <v>3</v>
@@ -59034,7 +59034,7 @@
         </is>
       </c>
       <c r="C3256" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3256" t="n">
         <v>3</v>
@@ -59052,7 +59052,7 @@
         </is>
       </c>
       <c r="C3257" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3257" t="n">
         <v>3</v>
@@ -59070,7 +59070,7 @@
         </is>
       </c>
       <c r="C3258" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3258" t="n">
         <v>3</v>
@@ -59088,7 +59088,7 @@
         </is>
       </c>
       <c r="C3259" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3259" t="n">
         <v>3</v>
@@ -59097,16 +59097,16 @@
     <row r="3260">
       <c r="A3260" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3260" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3260" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3260" t="n">
         <v>3</v>
@@ -59124,7 +59124,7 @@
         </is>
       </c>
       <c r="C3261" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3261" t="n">
         <v>3</v>
@@ -59142,7 +59142,7 @@
         </is>
       </c>
       <c r="C3262" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3262" t="n">
         <v>3</v>
@@ -59160,10 +59160,10 @@
         </is>
       </c>
       <c r="C3263" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3263" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3264">
@@ -59178,7 +59178,7 @@
         </is>
       </c>
       <c r="C3264" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3264" t="n">
         <v>2</v>
@@ -59196,7 +59196,7 @@
         </is>
       </c>
       <c r="C3265" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3265" t="n">
         <v>2</v>
@@ -59214,7 +59214,7 @@
         </is>
       </c>
       <c r="C3266" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3266" t="n">
         <v>2</v>
@@ -59223,16 +59223,16 @@
     <row r="3267">
       <c r="A3267" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3267" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3267" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3267" t="n">
         <v>2</v>
@@ -59250,10 +59250,10 @@
         </is>
       </c>
       <c r="C3268" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3268" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3269">
@@ -59268,7 +59268,7 @@
         </is>
       </c>
       <c r="C3269" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3269" t="n">
         <v>3</v>
@@ -59286,7 +59286,7 @@
         </is>
       </c>
       <c r="C3270" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3270" t="n">
         <v>3</v>
@@ -59304,7 +59304,7 @@
         </is>
       </c>
       <c r="C3271" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3271" t="n">
         <v>3</v>
@@ -59322,7 +59322,7 @@
         </is>
       </c>
       <c r="C3272" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3272" t="n">
         <v>3</v>
@@ -59340,7 +59340,7 @@
         </is>
       </c>
       <c r="C3273" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3273" t="n">
         <v>3</v>
@@ -59349,16 +59349,16 @@
     <row r="3274">
       <c r="A3274" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3274" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3274" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3274" t="n">
         <v>3</v>
@@ -59376,10 +59376,10 @@
         </is>
       </c>
       <c r="C3275" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3275" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3276">
@@ -59394,7 +59394,7 @@
         </is>
       </c>
       <c r="C3276" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3276" t="n">
         <v>4</v>
@@ -59412,10 +59412,10 @@
         </is>
       </c>
       <c r="C3277" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3277" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3278">
@@ -59430,7 +59430,7 @@
         </is>
       </c>
       <c r="C3278" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3278" t="n">
         <v>3</v>
@@ -59439,16 +59439,16 @@
     <row r="3279">
       <c r="A3279" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3279" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3279" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3279" t="n">
         <v>3</v>
@@ -59466,9 +59466,27 @@
         </is>
       </c>
       <c r="C3280" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3280" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3281">
+      <c r="A3281" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3281" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3281" t="n">
         <v>7</v>
       </c>
-      <c r="D3280" t="n">
+      <c r="D3281" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-03-22 07:06 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3350"/>
+  <dimension ref="A1:D3351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59979,19 +59979,19 @@
     <row r="3309">
       <c r="A3309" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/03/22</t>
         </is>
       </c>
       <c r="B3309" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3309" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3309" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3310">
@@ -60006,7 +60006,7 @@
         </is>
       </c>
       <c r="C3310" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3310" t="n">
         <v>3</v>
@@ -60024,7 +60024,7 @@
         </is>
       </c>
       <c r="C3311" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3311" t="n">
         <v>3</v>
@@ -60042,7 +60042,7 @@
         </is>
       </c>
       <c r="C3312" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3312" t="n">
         <v>3</v>
@@ -60051,16 +60051,16 @@
     <row r="3313">
       <c r="A3313" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3313" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3313" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3313" t="n">
         <v>3</v>
@@ -60078,7 +60078,7 @@
         </is>
       </c>
       <c r="C3314" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3314" t="n">
         <v>3</v>
@@ -60096,7 +60096,7 @@
         </is>
       </c>
       <c r="C3315" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3315" t="n">
         <v>3</v>
@@ -60114,7 +60114,7 @@
         </is>
       </c>
       <c r="C3316" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3316" t="n">
         <v>3</v>
@@ -60132,7 +60132,7 @@
         </is>
       </c>
       <c r="C3317" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3317" t="n">
         <v>3</v>
@@ -60150,7 +60150,7 @@
         </is>
       </c>
       <c r="C3318" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3318" t="n">
         <v>3</v>
@@ -60159,16 +60159,16 @@
     <row r="3319">
       <c r="A3319" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3319" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3319" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3319" t="n">
         <v>3</v>
@@ -60186,7 +60186,7 @@
         </is>
       </c>
       <c r="C3320" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3320" t="n">
         <v>3</v>
@@ -60204,7 +60204,7 @@
         </is>
       </c>
       <c r="C3321" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3321" t="n">
         <v>3</v>
@@ -60222,7 +60222,7 @@
         </is>
       </c>
       <c r="C3322" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3322" t="n">
         <v>3</v>
@@ -60240,7 +60240,7 @@
         </is>
       </c>
       <c r="C3323" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3323" t="n">
         <v>3</v>
@@ -60258,7 +60258,7 @@
         </is>
       </c>
       <c r="C3324" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3324" t="n">
         <v>3</v>
@@ -60267,16 +60267,16 @@
     <row r="3325">
       <c r="A3325" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3325" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3325" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3325" t="n">
         <v>3</v>
@@ -60294,7 +60294,7 @@
         </is>
       </c>
       <c r="C3326" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3326" t="n">
         <v>3</v>
@@ -60312,7 +60312,7 @@
         </is>
       </c>
       <c r="C3327" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3327" t="n">
         <v>3</v>
@@ -60330,7 +60330,7 @@
         </is>
       </c>
       <c r="C3328" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3328" t="n">
         <v>3</v>
@@ -60348,7 +60348,7 @@
         </is>
       </c>
       <c r="C3329" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3329" t="n">
         <v>3</v>
@@ -60357,16 +60357,16 @@
     <row r="3330">
       <c r="A3330" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3330" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3330" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3330" t="n">
         <v>3</v>
@@ -60384,7 +60384,7 @@
         </is>
       </c>
       <c r="C3331" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3331" t="n">
         <v>3</v>
@@ -60402,7 +60402,7 @@
         </is>
       </c>
       <c r="C3332" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3332" t="n">
         <v>3</v>
@@ -60420,10 +60420,10 @@
         </is>
       </c>
       <c r="C3333" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3333" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3334">
@@ -60438,7 +60438,7 @@
         </is>
       </c>
       <c r="C3334" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3334" t="n">
         <v>2</v>
@@ -60456,7 +60456,7 @@
         </is>
       </c>
       <c r="C3335" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3335" t="n">
         <v>2</v>
@@ -60474,7 +60474,7 @@
         </is>
       </c>
       <c r="C3336" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3336" t="n">
         <v>2</v>
@@ -60483,16 +60483,16 @@
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3337" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3337" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3337" t="n">
         <v>2</v>
@@ -60510,10 +60510,10 @@
         </is>
       </c>
       <c r="C3338" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3338" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3339">
@@ -60528,7 +60528,7 @@
         </is>
       </c>
       <c r="C3339" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3339" t="n">
         <v>3</v>
@@ -60546,7 +60546,7 @@
         </is>
       </c>
       <c r="C3340" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3340" t="n">
         <v>3</v>
@@ -60564,7 +60564,7 @@
         </is>
       </c>
       <c r="C3341" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3341" t="n">
         <v>3</v>
@@ -60582,7 +60582,7 @@
         </is>
       </c>
       <c r="C3342" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3342" t="n">
         <v>3</v>
@@ -60600,7 +60600,7 @@
         </is>
       </c>
       <c r="C3343" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3343" t="n">
         <v>3</v>
@@ -60609,16 +60609,16 @@
     <row r="3344">
       <c r="A3344" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3344" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3344" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3344" t="n">
         <v>3</v>
@@ -60636,10 +60636,10 @@
         </is>
       </c>
       <c r="C3345" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3345" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3346">
@@ -60654,7 +60654,7 @@
         </is>
       </c>
       <c r="C3346" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3346" t="n">
         <v>4</v>
@@ -60672,10 +60672,10 @@
         </is>
       </c>
       <c r="C3347" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3347" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3348">
@@ -60690,7 +60690,7 @@
         </is>
       </c>
       <c r="C3348" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3348" t="n">
         <v>3</v>
@@ -60699,16 +60699,16 @@
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3349" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3349" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3349" t="n">
         <v>3</v>
@@ -60726,9 +60726,27 @@
         </is>
       </c>
       <c r="C3350" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3350" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3351">
+      <c r="A3351" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3351" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3351" t="n">
         <v>7</v>
       </c>
-      <c r="D3350" t="n">
+      <c r="D3351" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-02 04:36 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3415"/>
+  <dimension ref="A1:D3416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61149,12 +61149,12 @@
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/02</t>
         </is>
       </c>
       <c r="B3374" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3374" t="n">
@@ -61176,7 +61176,7 @@
         </is>
       </c>
       <c r="C3375" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3375" t="n">
         <v>3</v>
@@ -61194,7 +61194,7 @@
         </is>
       </c>
       <c r="C3376" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3376" t="n">
         <v>3</v>
@@ -61212,7 +61212,7 @@
         </is>
       </c>
       <c r="C3377" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3377" t="n">
         <v>3</v>
@@ -61221,16 +61221,16 @@
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3378" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3378" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3378" t="n">
         <v>3</v>
@@ -61248,7 +61248,7 @@
         </is>
       </c>
       <c r="C3379" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3379" t="n">
         <v>3</v>
@@ -61266,7 +61266,7 @@
         </is>
       </c>
       <c r="C3380" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3380" t="n">
         <v>3</v>
@@ -61284,7 +61284,7 @@
         </is>
       </c>
       <c r="C3381" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3381" t="n">
         <v>3</v>
@@ -61302,7 +61302,7 @@
         </is>
       </c>
       <c r="C3382" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3382" t="n">
         <v>3</v>
@@ -61320,7 +61320,7 @@
         </is>
       </c>
       <c r="C3383" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3383" t="n">
         <v>3</v>
@@ -61329,16 +61329,16 @@
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3384" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3384" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3384" t="n">
         <v>3</v>
@@ -61356,7 +61356,7 @@
         </is>
       </c>
       <c r="C3385" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3385" t="n">
         <v>3</v>
@@ -61374,7 +61374,7 @@
         </is>
       </c>
       <c r="C3386" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3386" t="n">
         <v>3</v>
@@ -61392,7 +61392,7 @@
         </is>
       </c>
       <c r="C3387" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3387" t="n">
         <v>3</v>
@@ -61410,7 +61410,7 @@
         </is>
       </c>
       <c r="C3388" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3388" t="n">
         <v>3</v>
@@ -61428,7 +61428,7 @@
         </is>
       </c>
       <c r="C3389" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3389" t="n">
         <v>3</v>
@@ -61437,16 +61437,16 @@
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3390" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3390" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3390" t="n">
         <v>3</v>
@@ -61464,7 +61464,7 @@
         </is>
       </c>
       <c r="C3391" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3391" t="n">
         <v>3</v>
@@ -61482,7 +61482,7 @@
         </is>
       </c>
       <c r="C3392" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3392" t="n">
         <v>3</v>
@@ -61500,7 +61500,7 @@
         </is>
       </c>
       <c r="C3393" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3393" t="n">
         <v>3</v>
@@ -61518,7 +61518,7 @@
         </is>
       </c>
       <c r="C3394" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3394" t="n">
         <v>3</v>
@@ -61527,16 +61527,16 @@
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3395" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3395" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3395" t="n">
         <v>3</v>
@@ -61554,7 +61554,7 @@
         </is>
       </c>
       <c r="C3396" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3396" t="n">
         <v>3</v>
@@ -61572,7 +61572,7 @@
         </is>
       </c>
       <c r="C3397" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3397" t="n">
         <v>3</v>
@@ -61590,10 +61590,10 @@
         </is>
       </c>
       <c r="C3398" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3398" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3399">
@@ -61608,7 +61608,7 @@
         </is>
       </c>
       <c r="C3399" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3399" t="n">
         <v>2</v>
@@ -61626,7 +61626,7 @@
         </is>
       </c>
       <c r="C3400" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3400" t="n">
         <v>2</v>
@@ -61644,7 +61644,7 @@
         </is>
       </c>
       <c r="C3401" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3401" t="n">
         <v>2</v>
@@ -61653,16 +61653,16 @@
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3402" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3402" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3402" t="n">
         <v>2</v>
@@ -61680,10 +61680,10 @@
         </is>
       </c>
       <c r="C3403" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3403" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3404">
@@ -61698,7 +61698,7 @@
         </is>
       </c>
       <c r="C3404" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3404" t="n">
         <v>3</v>
@@ -61716,7 +61716,7 @@
         </is>
       </c>
       <c r="C3405" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3405" t="n">
         <v>3</v>
@@ -61734,7 +61734,7 @@
         </is>
       </c>
       <c r="C3406" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3406" t="n">
         <v>3</v>
@@ -61752,7 +61752,7 @@
         </is>
       </c>
       <c r="C3407" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3407" t="n">
         <v>3</v>
@@ -61770,7 +61770,7 @@
         </is>
       </c>
       <c r="C3408" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3408" t="n">
         <v>3</v>
@@ -61779,16 +61779,16 @@
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3409" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3409" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3409" t="n">
         <v>3</v>
@@ -61806,10 +61806,10 @@
         </is>
       </c>
       <c r="C3410" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3410" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3411">
@@ -61824,7 +61824,7 @@
         </is>
       </c>
       <c r="C3411" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3411" t="n">
         <v>4</v>
@@ -61842,10 +61842,10 @@
         </is>
       </c>
       <c r="C3412" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3412" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3413">
@@ -61860,7 +61860,7 @@
         </is>
       </c>
       <c r="C3413" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3413" t="n">
         <v>3</v>
@@ -61869,16 +61869,16 @@
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3414" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3414" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3414" t="n">
         <v>3</v>
@@ -61896,9 +61896,27 @@
         </is>
       </c>
       <c r="C3415" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3415" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3416" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3416" t="n">
         <v>7</v>
       </c>
-      <c r="D3415" t="n">
+      <c r="D3416" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-02 05:13 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3416"/>
+  <dimension ref="A1:D3417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61167,16 +61167,16 @@
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/02</t>
         </is>
       </c>
       <c r="B3375" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3375" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3375" t="n">
         <v>3</v>
@@ -61194,7 +61194,7 @@
         </is>
       </c>
       <c r="C3376" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3376" t="n">
         <v>3</v>
@@ -61212,7 +61212,7 @@
         </is>
       </c>
       <c r="C3377" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3377" t="n">
         <v>3</v>
@@ -61230,7 +61230,7 @@
         </is>
       </c>
       <c r="C3378" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3378" t="n">
         <v>3</v>
@@ -61239,16 +61239,16 @@
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3379" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3379" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3379" t="n">
         <v>3</v>
@@ -61266,7 +61266,7 @@
         </is>
       </c>
       <c r="C3380" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3380" t="n">
         <v>3</v>
@@ -61284,7 +61284,7 @@
         </is>
       </c>
       <c r="C3381" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3381" t="n">
         <v>3</v>
@@ -61302,7 +61302,7 @@
         </is>
       </c>
       <c r="C3382" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3382" t="n">
         <v>3</v>
@@ -61320,7 +61320,7 @@
         </is>
       </c>
       <c r="C3383" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3383" t="n">
         <v>3</v>
@@ -61338,7 +61338,7 @@
         </is>
       </c>
       <c r="C3384" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3384" t="n">
         <v>3</v>
@@ -61347,16 +61347,16 @@
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3385" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3385" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3385" t="n">
         <v>3</v>
@@ -61374,7 +61374,7 @@
         </is>
       </c>
       <c r="C3386" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3386" t="n">
         <v>3</v>
@@ -61392,7 +61392,7 @@
         </is>
       </c>
       <c r="C3387" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3387" t="n">
         <v>3</v>
@@ -61410,7 +61410,7 @@
         </is>
       </c>
       <c r="C3388" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3388" t="n">
         <v>3</v>
@@ -61428,7 +61428,7 @@
         </is>
       </c>
       <c r="C3389" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3389" t="n">
         <v>3</v>
@@ -61446,7 +61446,7 @@
         </is>
       </c>
       <c r="C3390" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3390" t="n">
         <v>3</v>
@@ -61455,16 +61455,16 @@
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3391" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3391" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3391" t="n">
         <v>3</v>
@@ -61482,7 +61482,7 @@
         </is>
       </c>
       <c r="C3392" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3392" t="n">
         <v>3</v>
@@ -61500,7 +61500,7 @@
         </is>
       </c>
       <c r="C3393" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3393" t="n">
         <v>3</v>
@@ -61518,7 +61518,7 @@
         </is>
       </c>
       <c r="C3394" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3394" t="n">
         <v>3</v>
@@ -61536,7 +61536,7 @@
         </is>
       </c>
       <c r="C3395" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3395" t="n">
         <v>3</v>
@@ -61545,16 +61545,16 @@
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3396" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3396" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3396" t="n">
         <v>3</v>
@@ -61572,7 +61572,7 @@
         </is>
       </c>
       <c r="C3397" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3397" t="n">
         <v>3</v>
@@ -61590,7 +61590,7 @@
         </is>
       </c>
       <c r="C3398" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3398" t="n">
         <v>3</v>
@@ -61608,10 +61608,10 @@
         </is>
       </c>
       <c r="C3399" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3399" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3400">
@@ -61626,7 +61626,7 @@
         </is>
       </c>
       <c r="C3400" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3400" t="n">
         <v>2</v>
@@ -61644,7 +61644,7 @@
         </is>
       </c>
       <c r="C3401" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3401" t="n">
         <v>2</v>
@@ -61662,7 +61662,7 @@
         </is>
       </c>
       <c r="C3402" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3402" t="n">
         <v>2</v>
@@ -61671,16 +61671,16 @@
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3403" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3403" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3403" t="n">
         <v>2</v>
@@ -61698,10 +61698,10 @@
         </is>
       </c>
       <c r="C3404" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3404" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3405">
@@ -61716,7 +61716,7 @@
         </is>
       </c>
       <c r="C3405" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3405" t="n">
         <v>3</v>
@@ -61734,7 +61734,7 @@
         </is>
       </c>
       <c r="C3406" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3406" t="n">
         <v>3</v>
@@ -61752,7 +61752,7 @@
         </is>
       </c>
       <c r="C3407" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3407" t="n">
         <v>3</v>
@@ -61770,7 +61770,7 @@
         </is>
       </c>
       <c r="C3408" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3408" t="n">
         <v>3</v>
@@ -61788,7 +61788,7 @@
         </is>
       </c>
       <c r="C3409" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3409" t="n">
         <v>3</v>
@@ -61797,16 +61797,16 @@
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3410" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3410" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3410" t="n">
         <v>3</v>
@@ -61824,10 +61824,10 @@
         </is>
       </c>
       <c r="C3411" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3411" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3412">
@@ -61842,7 +61842,7 @@
         </is>
       </c>
       <c r="C3412" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3412" t="n">
         <v>4</v>
@@ -61860,10 +61860,10 @@
         </is>
       </c>
       <c r="C3413" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3413" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3414">
@@ -61878,7 +61878,7 @@
         </is>
       </c>
       <c r="C3414" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3414" t="n">
         <v>3</v>
@@ -61887,16 +61887,16 @@
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3415" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3415" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3415" t="n">
         <v>3</v>
@@ -61914,9 +61914,27 @@
         </is>
       </c>
       <c r="C3416" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3416" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3417" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3417" t="n">
         <v>7</v>
       </c>
-      <c r="D3416" t="n">
+      <c r="D3417" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-04 07:14 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3431"/>
+  <dimension ref="A1:D3432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61437,16 +61437,16 @@
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/04</t>
         </is>
       </c>
       <c r="B3390" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3390" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3390" t="n">
         <v>3</v>
@@ -61464,7 +61464,7 @@
         </is>
       </c>
       <c r="C3391" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3391" t="n">
         <v>3</v>
@@ -61482,7 +61482,7 @@
         </is>
       </c>
       <c r="C3392" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3392" t="n">
         <v>3</v>
@@ -61500,7 +61500,7 @@
         </is>
       </c>
       <c r="C3393" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3393" t="n">
         <v>3</v>
@@ -61509,16 +61509,16 @@
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3394" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3394" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3394" t="n">
         <v>3</v>
@@ -61536,7 +61536,7 @@
         </is>
       </c>
       <c r="C3395" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3395" t="n">
         <v>3</v>
@@ -61554,7 +61554,7 @@
         </is>
       </c>
       <c r="C3396" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3396" t="n">
         <v>3</v>
@@ -61572,7 +61572,7 @@
         </is>
       </c>
       <c r="C3397" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3397" t="n">
         <v>3</v>
@@ -61590,7 +61590,7 @@
         </is>
       </c>
       <c r="C3398" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3398" t="n">
         <v>3</v>
@@ -61608,7 +61608,7 @@
         </is>
       </c>
       <c r="C3399" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3399" t="n">
         <v>3</v>
@@ -61617,16 +61617,16 @@
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3400" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3400" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3400" t="n">
         <v>3</v>
@@ -61644,7 +61644,7 @@
         </is>
       </c>
       <c r="C3401" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3401" t="n">
         <v>3</v>
@@ -61662,7 +61662,7 @@
         </is>
       </c>
       <c r="C3402" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3402" t="n">
         <v>3</v>
@@ -61680,7 +61680,7 @@
         </is>
       </c>
       <c r="C3403" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3403" t="n">
         <v>3</v>
@@ -61698,7 +61698,7 @@
         </is>
       </c>
       <c r="C3404" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3404" t="n">
         <v>3</v>
@@ -61716,7 +61716,7 @@
         </is>
       </c>
       <c r="C3405" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3405" t="n">
         <v>3</v>
@@ -61725,16 +61725,16 @@
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3406" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3406" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3406" t="n">
         <v>3</v>
@@ -61752,7 +61752,7 @@
         </is>
       </c>
       <c r="C3407" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3407" t="n">
         <v>3</v>
@@ -61770,7 +61770,7 @@
         </is>
       </c>
       <c r="C3408" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3408" t="n">
         <v>3</v>
@@ -61788,7 +61788,7 @@
         </is>
       </c>
       <c r="C3409" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3409" t="n">
         <v>3</v>
@@ -61806,7 +61806,7 @@
         </is>
       </c>
       <c r="C3410" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3410" t="n">
         <v>3</v>
@@ -61815,16 +61815,16 @@
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3411" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3411" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3411" t="n">
         <v>3</v>
@@ -61842,7 +61842,7 @@
         </is>
       </c>
       <c r="C3412" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3412" t="n">
         <v>3</v>
@@ -61860,7 +61860,7 @@
         </is>
       </c>
       <c r="C3413" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3413" t="n">
         <v>3</v>
@@ -61878,10 +61878,10 @@
         </is>
       </c>
       <c r="C3414" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3414" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3415">
@@ -61896,7 +61896,7 @@
         </is>
       </c>
       <c r="C3415" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3415" t="n">
         <v>2</v>
@@ -61914,7 +61914,7 @@
         </is>
       </c>
       <c r="C3416" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3416" t="n">
         <v>2</v>
@@ -61932,7 +61932,7 @@
         </is>
       </c>
       <c r="C3417" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3417" t="n">
         <v>2</v>
@@ -61941,16 +61941,16 @@
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3418" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3418" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3418" t="n">
         <v>2</v>
@@ -61968,10 +61968,10 @@
         </is>
       </c>
       <c r="C3419" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3419" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3420">
@@ -61986,7 +61986,7 @@
         </is>
       </c>
       <c r="C3420" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3420" t="n">
         <v>3</v>
@@ -62004,7 +62004,7 @@
         </is>
       </c>
       <c r="C3421" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3421" t="n">
         <v>3</v>
@@ -62022,7 +62022,7 @@
         </is>
       </c>
       <c r="C3422" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3422" t="n">
         <v>3</v>
@@ -62040,7 +62040,7 @@
         </is>
       </c>
       <c r="C3423" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3423" t="n">
         <v>3</v>
@@ -62058,7 +62058,7 @@
         </is>
       </c>
       <c r="C3424" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3424" t="n">
         <v>3</v>
@@ -62067,16 +62067,16 @@
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3425" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3425" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3425" t="n">
         <v>3</v>
@@ -62094,10 +62094,10 @@
         </is>
       </c>
       <c r="C3426" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3426" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3427">
@@ -62112,7 +62112,7 @@
         </is>
       </c>
       <c r="C3427" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3427" t="n">
         <v>4</v>
@@ -62130,10 +62130,10 @@
         </is>
       </c>
       <c r="C3428" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3428" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3429">
@@ -62148,7 +62148,7 @@
         </is>
       </c>
       <c r="C3429" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3429" t="n">
         <v>3</v>
@@ -62157,16 +62157,16 @@
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3430" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3430" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3430" t="n">
         <v>3</v>
@@ -62184,9 +62184,27 @@
         </is>
       </c>
       <c r="C3431" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3431" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3432">
+      <c r="A3432" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3432" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3432" t="n">
         <v>7</v>
       </c>
-      <c r="D3431" t="n">
+      <c r="D3432" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-09 08:44 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3461"/>
+  <dimension ref="A1:D3462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61977,16 +61977,16 @@
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/09</t>
         </is>
       </c>
       <c r="B3420" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3420" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D3420" t="n">
         <v>3</v>
@@ -62004,7 +62004,7 @@
         </is>
       </c>
       <c r="C3421" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3421" t="n">
         <v>3</v>
@@ -62022,7 +62022,7 @@
         </is>
       </c>
       <c r="C3422" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3422" t="n">
         <v>3</v>
@@ -62040,7 +62040,7 @@
         </is>
       </c>
       <c r="C3423" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3423" t="n">
         <v>3</v>
@@ -62049,16 +62049,16 @@
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3424" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3424" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3424" t="n">
         <v>3</v>
@@ -62076,7 +62076,7 @@
         </is>
       </c>
       <c r="C3425" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3425" t="n">
         <v>3</v>
@@ -62094,7 +62094,7 @@
         </is>
       </c>
       <c r="C3426" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3426" t="n">
         <v>3</v>
@@ -62112,7 +62112,7 @@
         </is>
       </c>
       <c r="C3427" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3427" t="n">
         <v>3</v>
@@ -62130,7 +62130,7 @@
         </is>
       </c>
       <c r="C3428" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3428" t="n">
         <v>3</v>
@@ -62148,7 +62148,7 @@
         </is>
       </c>
       <c r="C3429" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3429" t="n">
         <v>3</v>
@@ -62157,16 +62157,16 @@
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3430" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3430" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3430" t="n">
         <v>3</v>
@@ -62184,7 +62184,7 @@
         </is>
       </c>
       <c r="C3431" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3431" t="n">
         <v>3</v>
@@ -62202,7 +62202,7 @@
         </is>
       </c>
       <c r="C3432" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3432" t="n">
         <v>3</v>
@@ -62220,7 +62220,7 @@
         </is>
       </c>
       <c r="C3433" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3433" t="n">
         <v>3</v>
@@ -62238,7 +62238,7 @@
         </is>
       </c>
       <c r="C3434" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3434" t="n">
         <v>3</v>
@@ -62256,7 +62256,7 @@
         </is>
       </c>
       <c r="C3435" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3435" t="n">
         <v>3</v>
@@ -62265,16 +62265,16 @@
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3436" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3436" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3436" t="n">
         <v>3</v>
@@ -62292,7 +62292,7 @@
         </is>
       </c>
       <c r="C3437" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3437" t="n">
         <v>3</v>
@@ -62310,7 +62310,7 @@
         </is>
       </c>
       <c r="C3438" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3438" t="n">
         <v>3</v>
@@ -62328,7 +62328,7 @@
         </is>
       </c>
       <c r="C3439" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3439" t="n">
         <v>3</v>
@@ -62346,7 +62346,7 @@
         </is>
       </c>
       <c r="C3440" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3440" t="n">
         <v>3</v>
@@ -62355,16 +62355,16 @@
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3441" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3441" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3441" t="n">
         <v>3</v>
@@ -62382,7 +62382,7 @@
         </is>
       </c>
       <c r="C3442" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3442" t="n">
         <v>3</v>
@@ -62400,7 +62400,7 @@
         </is>
       </c>
       <c r="C3443" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3443" t="n">
         <v>3</v>
@@ -62418,10 +62418,10 @@
         </is>
       </c>
       <c r="C3444" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3444" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3445">
@@ -62436,7 +62436,7 @@
         </is>
       </c>
       <c r="C3445" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3445" t="n">
         <v>2</v>
@@ -62454,7 +62454,7 @@
         </is>
       </c>
       <c r="C3446" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3446" t="n">
         <v>2</v>
@@ -62472,7 +62472,7 @@
         </is>
       </c>
       <c r="C3447" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3447" t="n">
         <v>2</v>
@@ -62481,16 +62481,16 @@
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3448" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3448" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3448" t="n">
         <v>2</v>
@@ -62508,10 +62508,10 @@
         </is>
       </c>
       <c r="C3449" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3449" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3450">
@@ -62526,7 +62526,7 @@
         </is>
       </c>
       <c r="C3450" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3450" t="n">
         <v>3</v>
@@ -62544,7 +62544,7 @@
         </is>
       </c>
       <c r="C3451" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3451" t="n">
         <v>3</v>
@@ -62562,7 +62562,7 @@
         </is>
       </c>
       <c r="C3452" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3452" t="n">
         <v>3</v>
@@ -62580,7 +62580,7 @@
         </is>
       </c>
       <c r="C3453" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3453" t="n">
         <v>3</v>
@@ -62598,7 +62598,7 @@
         </is>
       </c>
       <c r="C3454" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3454" t="n">
         <v>3</v>
@@ -62607,16 +62607,16 @@
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3455" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3455" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3455" t="n">
         <v>3</v>
@@ -62634,10 +62634,10 @@
         </is>
       </c>
       <c r="C3456" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3456" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3457">
@@ -62652,7 +62652,7 @@
         </is>
       </c>
       <c r="C3457" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3457" t="n">
         <v>4</v>
@@ -62670,10 +62670,10 @@
         </is>
       </c>
       <c r="C3458" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3458" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3459">
@@ -62688,7 +62688,7 @@
         </is>
       </c>
       <c r="C3459" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3459" t="n">
         <v>3</v>
@@ -62697,16 +62697,16 @@
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3460" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3460" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3460" t="n">
         <v>3</v>
@@ -62724,9 +62724,27 @@
         </is>
       </c>
       <c r="C3461" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3461" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3462">
+      <c r="A3462" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3462" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3462" t="n">
         <v>7</v>
       </c>
-      <c r="D3461" t="n">
+      <c r="D3462" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-14 03:39 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3494"/>
+  <dimension ref="A1:D3495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62571,7 +62571,7 @@
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/14</t>
         </is>
       </c>
       <c r="B3453" t="inlineStr">
@@ -62580,10 +62580,10 @@
         </is>
       </c>
       <c r="C3453" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3453" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3454">
@@ -62598,7 +62598,7 @@
         </is>
       </c>
       <c r="C3454" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3454" t="n">
         <v>3</v>
@@ -62616,7 +62616,7 @@
         </is>
       </c>
       <c r="C3455" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3455" t="n">
         <v>3</v>
@@ -62634,7 +62634,7 @@
         </is>
       </c>
       <c r="C3456" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3456" t="n">
         <v>3</v>
@@ -62643,16 +62643,16 @@
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3457" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3457" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3457" t="n">
         <v>3</v>
@@ -62670,7 +62670,7 @@
         </is>
       </c>
       <c r="C3458" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3458" t="n">
         <v>3</v>
@@ -62688,7 +62688,7 @@
         </is>
       </c>
       <c r="C3459" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3459" t="n">
         <v>3</v>
@@ -62706,7 +62706,7 @@
         </is>
       </c>
       <c r="C3460" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3460" t="n">
         <v>3</v>
@@ -62724,7 +62724,7 @@
         </is>
       </c>
       <c r="C3461" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3461" t="n">
         <v>3</v>
@@ -62742,7 +62742,7 @@
         </is>
       </c>
       <c r="C3462" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3462" t="n">
         <v>3</v>
@@ -62751,16 +62751,16 @@
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3463" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3463" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3463" t="n">
         <v>3</v>
@@ -62778,7 +62778,7 @@
         </is>
       </c>
       <c r="C3464" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3464" t="n">
         <v>3</v>
@@ -62796,7 +62796,7 @@
         </is>
       </c>
       <c r="C3465" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3465" t="n">
         <v>3</v>
@@ -62814,7 +62814,7 @@
         </is>
       </c>
       <c r="C3466" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3466" t="n">
         <v>3</v>
@@ -62832,7 +62832,7 @@
         </is>
       </c>
       <c r="C3467" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3467" t="n">
         <v>3</v>
@@ -62850,7 +62850,7 @@
         </is>
       </c>
       <c r="C3468" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3468" t="n">
         <v>3</v>
@@ -62859,16 +62859,16 @@
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3469" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3469" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3469" t="n">
         <v>3</v>
@@ -62886,7 +62886,7 @@
         </is>
       </c>
       <c r="C3470" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3470" t="n">
         <v>3</v>
@@ -62904,7 +62904,7 @@
         </is>
       </c>
       <c r="C3471" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3471" t="n">
         <v>3</v>
@@ -62922,7 +62922,7 @@
         </is>
       </c>
       <c r="C3472" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3472" t="n">
         <v>3</v>
@@ -62940,7 +62940,7 @@
         </is>
       </c>
       <c r="C3473" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3473" t="n">
         <v>3</v>
@@ -62949,16 +62949,16 @@
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3474" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3474" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3474" t="n">
         <v>3</v>
@@ -62976,7 +62976,7 @@
         </is>
       </c>
       <c r="C3475" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3475" t="n">
         <v>3</v>
@@ -62994,7 +62994,7 @@
         </is>
       </c>
       <c r="C3476" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3476" t="n">
         <v>3</v>
@@ -63012,10 +63012,10 @@
         </is>
       </c>
       <c r="C3477" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3477" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3478">
@@ -63030,7 +63030,7 @@
         </is>
       </c>
       <c r="C3478" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3478" t="n">
         <v>2</v>
@@ -63048,7 +63048,7 @@
         </is>
       </c>
       <c r="C3479" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3479" t="n">
         <v>2</v>
@@ -63066,7 +63066,7 @@
         </is>
       </c>
       <c r="C3480" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3480" t="n">
         <v>2</v>
@@ -63075,16 +63075,16 @@
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3481" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3481" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3481" t="n">
         <v>2</v>
@@ -63102,10 +63102,10 @@
         </is>
       </c>
       <c r="C3482" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3482" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3483">
@@ -63120,7 +63120,7 @@
         </is>
       </c>
       <c r="C3483" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3483" t="n">
         <v>3</v>
@@ -63138,7 +63138,7 @@
         </is>
       </c>
       <c r="C3484" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3484" t="n">
         <v>3</v>
@@ -63156,7 +63156,7 @@
         </is>
       </c>
       <c r="C3485" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3485" t="n">
         <v>3</v>
@@ -63174,7 +63174,7 @@
         </is>
       </c>
       <c r="C3486" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3486" t="n">
         <v>3</v>
@@ -63192,7 +63192,7 @@
         </is>
       </c>
       <c r="C3487" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3487" t="n">
         <v>3</v>
@@ -63201,16 +63201,16 @@
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3488" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3488" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3488" t="n">
         <v>3</v>
@@ -63228,10 +63228,10 @@
         </is>
       </c>
       <c r="C3489" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3489" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3490">
@@ -63246,7 +63246,7 @@
         </is>
       </c>
       <c r="C3490" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3490" t="n">
         <v>4</v>
@@ -63264,10 +63264,10 @@
         </is>
       </c>
       <c r="C3491" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3491" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3492">
@@ -63282,7 +63282,7 @@
         </is>
       </c>
       <c r="C3492" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3492" t="n">
         <v>3</v>
@@ -63291,16 +63291,16 @@
     <row r="3493">
       <c r="A3493" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3493" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3493" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3493" t="n">
         <v>3</v>
@@ -63318,9 +63318,27 @@
         </is>
       </c>
       <c r="C3494" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3494" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3495">
+      <c r="A3495" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3495" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3495" t="n">
         <v>7</v>
       </c>
-      <c r="D3494" t="n">
+      <c r="D3495" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-14 08:50 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3496"/>
+  <dimension ref="A1:D3497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62607,7 +62607,7 @@
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/14</t>
         </is>
       </c>
       <c r="B3455" t="inlineStr">
@@ -62616,10 +62616,10 @@
         </is>
       </c>
       <c r="C3455" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D3455" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3456">
@@ -62634,7 +62634,7 @@
         </is>
       </c>
       <c r="C3456" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3456" t="n">
         <v>3</v>
@@ -62652,7 +62652,7 @@
         </is>
       </c>
       <c r="C3457" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3457" t="n">
         <v>3</v>
@@ -62670,7 +62670,7 @@
         </is>
       </c>
       <c r="C3458" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3458" t="n">
         <v>3</v>
@@ -62679,16 +62679,16 @@
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3459" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3459" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3459" t="n">
         <v>3</v>
@@ -62706,7 +62706,7 @@
         </is>
       </c>
       <c r="C3460" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3460" t="n">
         <v>3</v>
@@ -62724,7 +62724,7 @@
         </is>
       </c>
       <c r="C3461" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3461" t="n">
         <v>3</v>
@@ -62742,7 +62742,7 @@
         </is>
       </c>
       <c r="C3462" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3462" t="n">
         <v>3</v>
@@ -62760,7 +62760,7 @@
         </is>
       </c>
       <c r="C3463" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3463" t="n">
         <v>3</v>
@@ -62778,7 +62778,7 @@
         </is>
       </c>
       <c r="C3464" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3464" t="n">
         <v>3</v>
@@ -62787,16 +62787,16 @@
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3465" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3465" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3465" t="n">
         <v>3</v>
@@ -62814,7 +62814,7 @@
         </is>
       </c>
       <c r="C3466" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3466" t="n">
         <v>3</v>
@@ -62832,7 +62832,7 @@
         </is>
       </c>
       <c r="C3467" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3467" t="n">
         <v>3</v>
@@ -62850,7 +62850,7 @@
         </is>
       </c>
       <c r="C3468" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3468" t="n">
         <v>3</v>
@@ -62868,7 +62868,7 @@
         </is>
       </c>
       <c r="C3469" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3469" t="n">
         <v>3</v>
@@ -62886,7 +62886,7 @@
         </is>
       </c>
       <c r="C3470" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3470" t="n">
         <v>3</v>
@@ -62895,16 +62895,16 @@
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3471" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3471" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3471" t="n">
         <v>3</v>
@@ -62922,7 +62922,7 @@
         </is>
       </c>
       <c r="C3472" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3472" t="n">
         <v>3</v>
@@ -62940,7 +62940,7 @@
         </is>
       </c>
       <c r="C3473" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3473" t="n">
         <v>3</v>
@@ -62958,7 +62958,7 @@
         </is>
       </c>
       <c r="C3474" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3474" t="n">
         <v>3</v>
@@ -62976,7 +62976,7 @@
         </is>
       </c>
       <c r="C3475" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3475" t="n">
         <v>3</v>
@@ -62985,16 +62985,16 @@
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3476" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3476" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3476" t="n">
         <v>3</v>
@@ -63012,7 +63012,7 @@
         </is>
       </c>
       <c r="C3477" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3477" t="n">
         <v>3</v>
@@ -63030,7 +63030,7 @@
         </is>
       </c>
       <c r="C3478" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3478" t="n">
         <v>3</v>
@@ -63048,10 +63048,10 @@
         </is>
       </c>
       <c r="C3479" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3479" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3480">
@@ -63066,7 +63066,7 @@
         </is>
       </c>
       <c r="C3480" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3480" t="n">
         <v>2</v>
@@ -63084,7 +63084,7 @@
         </is>
       </c>
       <c r="C3481" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3481" t="n">
         <v>2</v>
@@ -63102,7 +63102,7 @@
         </is>
       </c>
       <c r="C3482" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3482" t="n">
         <v>2</v>
@@ -63111,16 +63111,16 @@
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3483" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3483" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3483" t="n">
         <v>2</v>
@@ -63138,10 +63138,10 @@
         </is>
       </c>
       <c r="C3484" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3484" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3485">
@@ -63156,7 +63156,7 @@
         </is>
       </c>
       <c r="C3485" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3485" t="n">
         <v>3</v>
@@ -63174,7 +63174,7 @@
         </is>
       </c>
       <c r="C3486" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3486" t="n">
         <v>3</v>
@@ -63192,7 +63192,7 @@
         </is>
       </c>
       <c r="C3487" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3487" t="n">
         <v>3</v>
@@ -63210,7 +63210,7 @@
         </is>
       </c>
       <c r="C3488" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3488" t="n">
         <v>3</v>
@@ -63228,7 +63228,7 @@
         </is>
       </c>
       <c r="C3489" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3489" t="n">
         <v>3</v>
@@ -63237,16 +63237,16 @@
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3490" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3490" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3490" t="n">
         <v>3</v>
@@ -63264,10 +63264,10 @@
         </is>
       </c>
       <c r="C3491" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3491" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3492">
@@ -63282,7 +63282,7 @@
         </is>
       </c>
       <c r="C3492" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3492" t="n">
         <v>4</v>
@@ -63300,10 +63300,10 @@
         </is>
       </c>
       <c r="C3493" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3493" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3494">
@@ -63318,7 +63318,7 @@
         </is>
       </c>
       <c r="C3494" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3494" t="n">
         <v>3</v>
@@ -63327,16 +63327,16 @@
     <row r="3495">
       <c r="A3495" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3495" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3495" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3495" t="n">
         <v>3</v>
@@ -63354,9 +63354,27 @@
         </is>
       </c>
       <c r="C3496" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3496" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3497">
+      <c r="A3497" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3497" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3497" t="n">
         <v>7</v>
       </c>
-      <c r="D3496" t="n">
+      <c r="D3497" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-04-21 03:44 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3542"/>
+  <dimension ref="A1:D3543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63435,7 +63435,7 @@
     <row r="3501">
       <c r="A3501" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/04/21</t>
         </is>
       </c>
       <c r="B3501" t="inlineStr">
@@ -63444,10 +63444,10 @@
         </is>
       </c>
       <c r="C3501" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3501" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3502">
@@ -63462,7 +63462,7 @@
         </is>
       </c>
       <c r="C3502" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3502" t="n">
         <v>3</v>
@@ -63480,7 +63480,7 @@
         </is>
       </c>
       <c r="C3503" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3503" t="n">
         <v>3</v>
@@ -63498,7 +63498,7 @@
         </is>
       </c>
       <c r="C3504" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3504" t="n">
         <v>3</v>
@@ -63507,16 +63507,16 @@
     <row r="3505">
       <c r="A3505" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3505" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3505" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3505" t="n">
         <v>3</v>
@@ -63534,7 +63534,7 @@
         </is>
       </c>
       <c r="C3506" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3506" t="n">
         <v>3</v>
@@ -63552,7 +63552,7 @@
         </is>
       </c>
       <c r="C3507" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3507" t="n">
         <v>3</v>
@@ -63570,7 +63570,7 @@
         </is>
       </c>
       <c r="C3508" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3508" t="n">
         <v>3</v>
@@ -63588,7 +63588,7 @@
         </is>
       </c>
       <c r="C3509" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3509" t="n">
         <v>3</v>
@@ -63606,7 +63606,7 @@
         </is>
       </c>
       <c r="C3510" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3510" t="n">
         <v>3</v>
@@ -63615,16 +63615,16 @@
     <row r="3511">
       <c r="A3511" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3511" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3511" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3511" t="n">
         <v>3</v>
@@ -63642,7 +63642,7 @@
         </is>
       </c>
       <c r="C3512" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3512" t="n">
         <v>3</v>
@@ -63660,7 +63660,7 @@
         </is>
       </c>
       <c r="C3513" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3513" t="n">
         <v>3</v>
@@ -63678,7 +63678,7 @@
         </is>
       </c>
       <c r="C3514" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3514" t="n">
         <v>3</v>
@@ -63696,7 +63696,7 @@
         </is>
       </c>
       <c r="C3515" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3515" t="n">
         <v>3</v>
@@ -63714,7 +63714,7 @@
         </is>
       </c>
       <c r="C3516" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3516" t="n">
         <v>3</v>
@@ -63723,16 +63723,16 @@
     <row r="3517">
       <c r="A3517" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3517" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3517" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3517" t="n">
         <v>3</v>
@@ -63750,7 +63750,7 @@
         </is>
       </c>
       <c r="C3518" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3518" t="n">
         <v>3</v>
@@ -63768,7 +63768,7 @@
         </is>
       </c>
       <c r="C3519" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3519" t="n">
         <v>3</v>
@@ -63786,7 +63786,7 @@
         </is>
       </c>
       <c r="C3520" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3520" t="n">
         <v>3</v>
@@ -63804,7 +63804,7 @@
         </is>
       </c>
       <c r="C3521" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3521" t="n">
         <v>3</v>
@@ -63813,16 +63813,16 @@
     <row r="3522">
       <c r="A3522" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3522" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3522" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3522" t="n">
         <v>3</v>
@@ -63840,7 +63840,7 @@
         </is>
       </c>
       <c r="C3523" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3523" t="n">
         <v>3</v>
@@ -63858,7 +63858,7 @@
         </is>
       </c>
       <c r="C3524" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3524" t="n">
         <v>3</v>
@@ -63876,10 +63876,10 @@
         </is>
       </c>
       <c r="C3525" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3525" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3526">
@@ -63894,7 +63894,7 @@
         </is>
       </c>
       <c r="C3526" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3526" t="n">
         <v>2</v>
@@ -63912,7 +63912,7 @@
         </is>
       </c>
       <c r="C3527" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3527" t="n">
         <v>2</v>
@@ -63930,7 +63930,7 @@
         </is>
       </c>
       <c r="C3528" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3528" t="n">
         <v>2</v>
@@ -63939,16 +63939,16 @@
     <row r="3529">
       <c r="A3529" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3529" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3529" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3529" t="n">
         <v>2</v>
@@ -63966,10 +63966,10 @@
         </is>
       </c>
       <c r="C3530" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3530" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3531">
@@ -63984,7 +63984,7 @@
         </is>
       </c>
       <c r="C3531" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3531" t="n">
         <v>3</v>
@@ -64002,7 +64002,7 @@
         </is>
       </c>
       <c r="C3532" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3532" t="n">
         <v>3</v>
@@ -64020,7 +64020,7 @@
         </is>
       </c>
       <c r="C3533" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3533" t="n">
         <v>3</v>
@@ -64038,7 +64038,7 @@
         </is>
       </c>
       <c r="C3534" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3534" t="n">
         <v>3</v>
@@ -64056,7 +64056,7 @@
         </is>
       </c>
       <c r="C3535" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3535" t="n">
         <v>3</v>
@@ -64065,16 +64065,16 @@
     <row r="3536">
       <c r="A3536" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3536" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3536" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3536" t="n">
         <v>3</v>
@@ -64092,10 +64092,10 @@
         </is>
       </c>
       <c r="C3537" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3537" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3538">
@@ -64110,7 +64110,7 @@
         </is>
       </c>
       <c r="C3538" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3538" t="n">
         <v>4</v>
@@ -64128,10 +64128,10 @@
         </is>
       </c>
       <c r="C3539" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3539" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3540">
@@ -64146,7 +64146,7 @@
         </is>
       </c>
       <c r="C3540" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3540" t="n">
         <v>3</v>
@@ -64155,16 +64155,16 @@
     <row r="3541">
       <c r="A3541" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3541" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3541" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3541" t="n">
         <v>3</v>
@@ -64182,9 +64182,27 @@
         </is>
       </c>
       <c r="C3542" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3542" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3543">
+      <c r="A3543" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3543" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3543" t="n">
         <v>7</v>
       </c>
-      <c r="D3542" t="n">
+      <c r="D3543" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-05-03 04:09 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3619"/>
+  <dimension ref="A1:D3620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64821,19 +64821,19 @@
     <row r="3578">
       <c r="A3578" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/05/03</t>
         </is>
       </c>
       <c r="B3578" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3578" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3578" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3579">
@@ -64848,7 +64848,7 @@
         </is>
       </c>
       <c r="C3579" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3579" t="n">
         <v>3</v>
@@ -64866,7 +64866,7 @@
         </is>
       </c>
       <c r="C3580" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3580" t="n">
         <v>3</v>
@@ -64884,7 +64884,7 @@
         </is>
       </c>
       <c r="C3581" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3581" t="n">
         <v>3</v>
@@ -64893,16 +64893,16 @@
     <row r="3582">
       <c r="A3582" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3582" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3582" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3582" t="n">
         <v>3</v>
@@ -64920,7 +64920,7 @@
         </is>
       </c>
       <c r="C3583" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3583" t="n">
         <v>3</v>
@@ -64938,7 +64938,7 @@
         </is>
       </c>
       <c r="C3584" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3584" t="n">
         <v>3</v>
@@ -64956,7 +64956,7 @@
         </is>
       </c>
       <c r="C3585" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3585" t="n">
         <v>3</v>
@@ -64974,7 +64974,7 @@
         </is>
       </c>
       <c r="C3586" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3586" t="n">
         <v>3</v>
@@ -64992,7 +64992,7 @@
         </is>
       </c>
       <c r="C3587" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3587" t="n">
         <v>3</v>
@@ -65001,16 +65001,16 @@
     <row r="3588">
       <c r="A3588" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3588" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3588" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3588" t="n">
         <v>3</v>
@@ -65028,7 +65028,7 @@
         </is>
       </c>
       <c r="C3589" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3589" t="n">
         <v>3</v>
@@ -65046,7 +65046,7 @@
         </is>
       </c>
       <c r="C3590" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3590" t="n">
         <v>3</v>
@@ -65064,7 +65064,7 @@
         </is>
       </c>
       <c r="C3591" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3591" t="n">
         <v>3</v>
@@ -65082,7 +65082,7 @@
         </is>
       </c>
       <c r="C3592" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3592" t="n">
         <v>3</v>
@@ -65100,7 +65100,7 @@
         </is>
       </c>
       <c r="C3593" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3593" t="n">
         <v>3</v>
@@ -65109,16 +65109,16 @@
     <row r="3594">
       <c r="A3594" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3594" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3594" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3594" t="n">
         <v>3</v>
@@ -65136,7 +65136,7 @@
         </is>
       </c>
       <c r="C3595" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3595" t="n">
         <v>3</v>
@@ -65154,7 +65154,7 @@
         </is>
       </c>
       <c r="C3596" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3596" t="n">
         <v>3</v>
@@ -65172,7 +65172,7 @@
         </is>
       </c>
       <c r="C3597" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3597" t="n">
         <v>3</v>
@@ -65190,7 +65190,7 @@
         </is>
       </c>
       <c r="C3598" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3598" t="n">
         <v>3</v>
@@ -65199,16 +65199,16 @@
     <row r="3599">
       <c r="A3599" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3599" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3599" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3599" t="n">
         <v>3</v>
@@ -65226,7 +65226,7 @@
         </is>
       </c>
       <c r="C3600" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3600" t="n">
         <v>3</v>
@@ -65244,7 +65244,7 @@
         </is>
       </c>
       <c r="C3601" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3601" t="n">
         <v>3</v>
@@ -65262,10 +65262,10 @@
         </is>
       </c>
       <c r="C3602" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3602" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3603">
@@ -65280,7 +65280,7 @@
         </is>
       </c>
       <c r="C3603" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3603" t="n">
         <v>2</v>
@@ -65298,7 +65298,7 @@
         </is>
       </c>
       <c r="C3604" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3604" t="n">
         <v>2</v>
@@ -65316,7 +65316,7 @@
         </is>
       </c>
       <c r="C3605" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3605" t="n">
         <v>2</v>
@@ -65325,16 +65325,16 @@
     <row r="3606">
       <c r="A3606" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3606" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3606" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3606" t="n">
         <v>2</v>
@@ -65352,10 +65352,10 @@
         </is>
       </c>
       <c r="C3607" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3607" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3608">
@@ -65370,7 +65370,7 @@
         </is>
       </c>
       <c r="C3608" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3608" t="n">
         <v>3</v>
@@ -65388,7 +65388,7 @@
         </is>
       </c>
       <c r="C3609" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3609" t="n">
         <v>3</v>
@@ -65406,7 +65406,7 @@
         </is>
       </c>
       <c r="C3610" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3610" t="n">
         <v>3</v>
@@ -65424,7 +65424,7 @@
         </is>
       </c>
       <c r="C3611" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3611" t="n">
         <v>3</v>
@@ -65442,7 +65442,7 @@
         </is>
       </c>
       <c r="C3612" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3612" t="n">
         <v>3</v>
@@ -65451,16 +65451,16 @@
     <row r="3613">
       <c r="A3613" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3613" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3613" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3613" t="n">
         <v>3</v>
@@ -65478,10 +65478,10 @@
         </is>
       </c>
       <c r="C3614" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3614" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3615">
@@ -65496,7 +65496,7 @@
         </is>
       </c>
       <c r="C3615" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3615" t="n">
         <v>4</v>
@@ -65514,10 +65514,10 @@
         </is>
       </c>
       <c r="C3616" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3616" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3617">
@@ -65532,7 +65532,7 @@
         </is>
       </c>
       <c r="C3617" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3617" t="n">
         <v>3</v>
@@ -65541,16 +65541,16 @@
     <row r="3618">
       <c r="A3618" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3618" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3618" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3618" t="n">
         <v>3</v>
@@ -65568,9 +65568,27 @@
         </is>
       </c>
       <c r="C3619" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3619" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3620">
+      <c r="A3620" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3620" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3620" t="n">
         <v>7</v>
       </c>
-      <c r="D3619" t="n">
+      <c r="D3620" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-05-28 12:41 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3781"/>
+  <dimension ref="A1:D3782"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67737,19 +67737,19 @@
     <row r="3740">
       <c r="A3740" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/05/28</t>
         </is>
       </c>
       <c r="B3740" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3740" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D3740" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3741">
@@ -67764,7 +67764,7 @@
         </is>
       </c>
       <c r="C3741" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3741" t="n">
         <v>3</v>
@@ -67782,7 +67782,7 @@
         </is>
       </c>
       <c r="C3742" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3742" t="n">
         <v>3</v>
@@ -67800,7 +67800,7 @@
         </is>
       </c>
       <c r="C3743" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D3743" t="n">
         <v>3</v>
@@ -67809,16 +67809,16 @@
     <row r="3744">
       <c r="A3744" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B3744" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C3744" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D3744" t="n">
         <v>3</v>
@@ -67836,7 +67836,7 @@
         </is>
       </c>
       <c r="C3745" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3745" t="n">
         <v>3</v>
@@ -67854,7 +67854,7 @@
         </is>
       </c>
       <c r="C3746" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3746" t="n">
         <v>3</v>
@@ -67872,7 +67872,7 @@
         </is>
       </c>
       <c r="C3747" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3747" t="n">
         <v>3</v>
@@ -67890,7 +67890,7 @@
         </is>
       </c>
       <c r="C3748" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3748" t="n">
         <v>3</v>
@@ -67908,7 +67908,7 @@
         </is>
       </c>
       <c r="C3749" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3749" t="n">
         <v>3</v>
@@ -67917,16 +67917,16 @@
     <row r="3750">
       <c r="A3750" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B3750" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C3750" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3750" t="n">
         <v>3</v>
@@ -67944,7 +67944,7 @@
         </is>
       </c>
       <c r="C3751" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D3751" t="n">
         <v>3</v>
@@ -67962,7 +67962,7 @@
         </is>
       </c>
       <c r="C3752" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3752" t="n">
         <v>3</v>
@@ -67980,7 +67980,7 @@
         </is>
       </c>
       <c r="C3753" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3753" t="n">
         <v>3</v>
@@ -67998,7 +67998,7 @@
         </is>
       </c>
       <c r="C3754" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3754" t="n">
         <v>3</v>
@@ -68016,7 +68016,7 @@
         </is>
       </c>
       <c r="C3755" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D3755" t="n">
         <v>3</v>
@@ -68025,16 +68025,16 @@
     <row r="3756">
       <c r="A3756" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B3756" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C3756" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3756" t="n">
         <v>3</v>
@@ -68052,7 +68052,7 @@
         </is>
       </c>
       <c r="C3757" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3757" t="n">
         <v>3</v>
@@ -68070,7 +68070,7 @@
         </is>
       </c>
       <c r="C3758" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3758" t="n">
         <v>3</v>
@@ -68088,7 +68088,7 @@
         </is>
       </c>
       <c r="C3759" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3759" t="n">
         <v>3</v>
@@ -68106,7 +68106,7 @@
         </is>
       </c>
       <c r="C3760" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3760" t="n">
         <v>3</v>
@@ -68115,16 +68115,16 @@
     <row r="3761">
       <c r="A3761" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B3761" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C3761" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D3761" t="n">
         <v>3</v>
@@ -68142,7 +68142,7 @@
         </is>
       </c>
       <c r="C3762" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3762" t="n">
         <v>3</v>
@@ -68160,7 +68160,7 @@
         </is>
       </c>
       <c r="C3763" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3763" t="n">
         <v>3</v>
@@ -68178,10 +68178,10 @@
         </is>
       </c>
       <c r="C3764" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3764" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3765">
@@ -68196,7 +68196,7 @@
         </is>
       </c>
       <c r="C3765" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3765" t="n">
         <v>2</v>
@@ -68214,7 +68214,7 @@
         </is>
       </c>
       <c r="C3766" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3766" t="n">
         <v>2</v>
@@ -68232,7 +68232,7 @@
         </is>
       </c>
       <c r="C3767" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3767" t="n">
         <v>2</v>
@@ -68241,16 +68241,16 @@
     <row r="3768">
       <c r="A3768" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B3768" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3768" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3768" t="n">
         <v>2</v>
@@ -68268,10 +68268,10 @@
         </is>
       </c>
       <c r="C3769" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3769" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3770">
@@ -68286,7 +68286,7 @@
         </is>
       </c>
       <c r="C3770" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3770" t="n">
         <v>3</v>
@@ -68304,7 +68304,7 @@
         </is>
       </c>
       <c r="C3771" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3771" t="n">
         <v>3</v>
@@ -68322,7 +68322,7 @@
         </is>
       </c>
       <c r="C3772" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D3772" t="n">
         <v>3</v>
@@ -68340,7 +68340,7 @@
         </is>
       </c>
       <c r="C3773" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3773" t="n">
         <v>3</v>
@@ -68358,7 +68358,7 @@
         </is>
       </c>
       <c r="C3774" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3774" t="n">
         <v>3</v>
@@ -68367,16 +68367,16 @@
     <row r="3775">
       <c r="A3775" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B3775" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C3775" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D3775" t="n">
         <v>3</v>
@@ -68394,10 +68394,10 @@
         </is>
       </c>
       <c r="C3776" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3776" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3777">
@@ -68412,7 +68412,7 @@
         </is>
       </c>
       <c r="C3777" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3777" t="n">
         <v>4</v>
@@ -68430,10 +68430,10 @@
         </is>
       </c>
       <c r="C3778" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D3778" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3779">
@@ -68448,7 +68448,7 @@
         </is>
       </c>
       <c r="C3779" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D3779" t="n">
         <v>3</v>
@@ -68457,16 +68457,16 @@
     <row r="3780">
       <c r="A3780" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B3780" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C3780" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D3780" t="n">
         <v>3</v>
@@ -68484,9 +68484,27 @@
         </is>
       </c>
       <c r="C3781" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3781" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3782">
+      <c r="A3782" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B3782" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C3782" t="n">
         <v>7</v>
       </c>
-      <c r="D3781" t="n">
+      <c r="D3782" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-13 07:48 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4482"/>
+  <dimension ref="A1:D4483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80355,19 +80355,19 @@
     <row r="4441">
       <c r="A4441" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/13</t>
         </is>
       </c>
       <c r="B4441" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4441" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D4441" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4442">
@@ -80382,7 +80382,7 @@
         </is>
       </c>
       <c r="C4442" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4442" t="n">
         <v>3</v>
@@ -80400,7 +80400,7 @@
         </is>
       </c>
       <c r="C4443" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4443" t="n">
         <v>3</v>
@@ -80418,7 +80418,7 @@
         </is>
       </c>
       <c r="C4444" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4444" t="n">
         <v>3</v>
@@ -80427,16 +80427,16 @@
     <row r="4445">
       <c r="A4445" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4445" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4445" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4445" t="n">
         <v>3</v>
@@ -80454,7 +80454,7 @@
         </is>
       </c>
       <c r="C4446" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4446" t="n">
         <v>3</v>
@@ -80472,7 +80472,7 @@
         </is>
       </c>
       <c r="C4447" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4447" t="n">
         <v>3</v>
@@ -80490,7 +80490,7 @@
         </is>
       </c>
       <c r="C4448" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4448" t="n">
         <v>3</v>
@@ -80508,7 +80508,7 @@
         </is>
       </c>
       <c r="C4449" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4449" t="n">
         <v>3</v>
@@ -80526,7 +80526,7 @@
         </is>
       </c>
       <c r="C4450" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4450" t="n">
         <v>3</v>
@@ -80535,16 +80535,16 @@
     <row r="4451">
       <c r="A4451" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4451" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4451" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4451" t="n">
         <v>3</v>
@@ -80562,7 +80562,7 @@
         </is>
       </c>
       <c r="C4452" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4452" t="n">
         <v>3</v>
@@ -80580,7 +80580,7 @@
         </is>
       </c>
       <c r="C4453" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4453" t="n">
         <v>3</v>
@@ -80598,7 +80598,7 @@
         </is>
       </c>
       <c r="C4454" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4454" t="n">
         <v>3</v>
@@ -80616,7 +80616,7 @@
         </is>
       </c>
       <c r="C4455" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4455" t="n">
         <v>3</v>
@@ -80634,7 +80634,7 @@
         </is>
       </c>
       <c r="C4456" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4456" t="n">
         <v>3</v>
@@ -80643,16 +80643,16 @@
     <row r="4457">
       <c r="A4457" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4457" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4457" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4457" t="n">
         <v>3</v>
@@ -80670,7 +80670,7 @@
         </is>
       </c>
       <c r="C4458" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4458" t="n">
         <v>3</v>
@@ -80688,7 +80688,7 @@
         </is>
       </c>
       <c r="C4459" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4459" t="n">
         <v>3</v>
@@ -80706,7 +80706,7 @@
         </is>
       </c>
       <c r="C4460" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4460" t="n">
         <v>3</v>
@@ -80724,7 +80724,7 @@
         </is>
       </c>
       <c r="C4461" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4461" t="n">
         <v>3</v>
@@ -80733,16 +80733,16 @@
     <row r="4462">
       <c r="A4462" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4462" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4462" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4462" t="n">
         <v>3</v>
@@ -80760,7 +80760,7 @@
         </is>
       </c>
       <c r="C4463" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4463" t="n">
         <v>3</v>
@@ -80778,7 +80778,7 @@
         </is>
       </c>
       <c r="C4464" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4464" t="n">
         <v>3</v>
@@ -80796,10 +80796,10 @@
         </is>
       </c>
       <c r="C4465" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4465" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4466">
@@ -80814,7 +80814,7 @@
         </is>
       </c>
       <c r="C4466" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4466" t="n">
         <v>2</v>
@@ -80832,7 +80832,7 @@
         </is>
       </c>
       <c r="C4467" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4467" t="n">
         <v>2</v>
@@ -80850,7 +80850,7 @@
         </is>
       </c>
       <c r="C4468" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4468" t="n">
         <v>2</v>
@@ -80859,16 +80859,16 @@
     <row r="4469">
       <c r="A4469" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4469" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4469" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4469" t="n">
         <v>2</v>
@@ -80886,10 +80886,10 @@
         </is>
       </c>
       <c r="C4470" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4470" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4471">
@@ -80904,7 +80904,7 @@
         </is>
       </c>
       <c r="C4471" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4471" t="n">
         <v>3</v>
@@ -80922,7 +80922,7 @@
         </is>
       </c>
       <c r="C4472" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4472" t="n">
         <v>3</v>
@@ -80940,7 +80940,7 @@
         </is>
       </c>
       <c r="C4473" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4473" t="n">
         <v>3</v>
@@ -80958,7 +80958,7 @@
         </is>
       </c>
       <c r="C4474" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4474" t="n">
         <v>3</v>
@@ -80976,7 +80976,7 @@
         </is>
       </c>
       <c r="C4475" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4475" t="n">
         <v>3</v>
@@ -80985,16 +80985,16 @@
     <row r="4476">
       <c r="A4476" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4476" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4476" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4476" t="n">
         <v>3</v>
@@ -81012,10 +81012,10 @@
         </is>
       </c>
       <c r="C4477" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4477" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4478">
@@ -81030,7 +81030,7 @@
         </is>
       </c>
       <c r="C4478" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4478" t="n">
         <v>4</v>
@@ -81048,10 +81048,10 @@
         </is>
       </c>
       <c r="C4479" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4479" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4480">
@@ -81066,7 +81066,7 @@
         </is>
       </c>
       <c r="C4480" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4480" t="n">
         <v>3</v>
@@ -81075,16 +81075,16 @@
     <row r="4481">
       <c r="A4481" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4481" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4481" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4481" t="n">
         <v>3</v>
@@ -81102,9 +81102,27 @@
         </is>
       </c>
       <c r="C4482" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4482" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4483">
+      <c r="A4483" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4483" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4483" t="n">
         <v>7</v>
       </c>
-      <c r="D4482" t="n">
+      <c r="D4483" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-08-29 08:57 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4596"/>
+  <dimension ref="A1:D4597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82407,19 +82407,19 @@
     <row r="4555">
       <c r="A4555" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/29</t>
         </is>
       </c>
       <c r="B4555" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4555" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D4555" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4556">
@@ -82434,7 +82434,7 @@
         </is>
       </c>
       <c r="C4556" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4556" t="n">
         <v>3</v>
@@ -82452,7 +82452,7 @@
         </is>
       </c>
       <c r="C4557" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4557" t="n">
         <v>3</v>
@@ -82470,7 +82470,7 @@
         </is>
       </c>
       <c r="C4558" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4558" t="n">
         <v>3</v>
@@ -82479,16 +82479,16 @@
     <row r="4559">
       <c r="A4559" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4559" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4559" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4559" t="n">
         <v>3</v>
@@ -82506,7 +82506,7 @@
         </is>
       </c>
       <c r="C4560" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4560" t="n">
         <v>3</v>
@@ -82524,7 +82524,7 @@
         </is>
       </c>
       <c r="C4561" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4561" t="n">
         <v>3</v>
@@ -82542,7 +82542,7 @@
         </is>
       </c>
       <c r="C4562" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4562" t="n">
         <v>3</v>
@@ -82560,7 +82560,7 @@
         </is>
       </c>
       <c r="C4563" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4563" t="n">
         <v>3</v>
@@ -82578,7 +82578,7 @@
         </is>
       </c>
       <c r="C4564" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4564" t="n">
         <v>3</v>
@@ -82587,16 +82587,16 @@
     <row r="4565">
       <c r="A4565" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4565" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4565" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4565" t="n">
         <v>3</v>
@@ -82614,7 +82614,7 @@
         </is>
       </c>
       <c r="C4566" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4566" t="n">
         <v>3</v>
@@ -82632,7 +82632,7 @@
         </is>
       </c>
       <c r="C4567" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4567" t="n">
         <v>3</v>
@@ -82650,7 +82650,7 @@
         </is>
       </c>
       <c r="C4568" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4568" t="n">
         <v>3</v>
@@ -82668,7 +82668,7 @@
         </is>
       </c>
       <c r="C4569" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4569" t="n">
         <v>3</v>
@@ -82686,7 +82686,7 @@
         </is>
       </c>
       <c r="C4570" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4570" t="n">
         <v>3</v>
@@ -82695,16 +82695,16 @@
     <row r="4571">
       <c r="A4571" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4571" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4571" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4571" t="n">
         <v>3</v>
@@ -82722,7 +82722,7 @@
         </is>
       </c>
       <c r="C4572" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4572" t="n">
         <v>3</v>
@@ -82740,7 +82740,7 @@
         </is>
       </c>
       <c r="C4573" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4573" t="n">
         <v>3</v>
@@ -82758,7 +82758,7 @@
         </is>
       </c>
       <c r="C4574" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4574" t="n">
         <v>3</v>
@@ -82776,7 +82776,7 @@
         </is>
       </c>
       <c r="C4575" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4575" t="n">
         <v>3</v>
@@ -82785,16 +82785,16 @@
     <row r="4576">
       <c r="A4576" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4576" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4576" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4576" t="n">
         <v>3</v>
@@ -82812,7 +82812,7 @@
         </is>
       </c>
       <c r="C4577" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4577" t="n">
         <v>3</v>
@@ -82830,7 +82830,7 @@
         </is>
       </c>
       <c r="C4578" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4578" t="n">
         <v>3</v>
@@ -82848,10 +82848,10 @@
         </is>
       </c>
       <c r="C4579" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4579" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4580">
@@ -82866,7 +82866,7 @@
         </is>
       </c>
       <c r="C4580" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4580" t="n">
         <v>2</v>
@@ -82884,7 +82884,7 @@
         </is>
       </c>
       <c r="C4581" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4581" t="n">
         <v>2</v>
@@ -82902,7 +82902,7 @@
         </is>
       </c>
       <c r="C4582" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4582" t="n">
         <v>2</v>
@@ -82911,16 +82911,16 @@
     <row r="4583">
       <c r="A4583" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4583" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4583" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4583" t="n">
         <v>2</v>
@@ -82938,10 +82938,10 @@
         </is>
       </c>
       <c r="C4584" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4584" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4585">
@@ -82956,7 +82956,7 @@
         </is>
       </c>
       <c r="C4585" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4585" t="n">
         <v>3</v>
@@ -82974,7 +82974,7 @@
         </is>
       </c>
       <c r="C4586" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4586" t="n">
         <v>3</v>
@@ -82992,7 +82992,7 @@
         </is>
       </c>
       <c r="C4587" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4587" t="n">
         <v>3</v>
@@ -83010,7 +83010,7 @@
         </is>
       </c>
       <c r="C4588" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4588" t="n">
         <v>3</v>
@@ -83028,7 +83028,7 @@
         </is>
       </c>
       <c r="C4589" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4589" t="n">
         <v>3</v>
@@ -83037,16 +83037,16 @@
     <row r="4590">
       <c r="A4590" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4590" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4590" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4590" t="n">
         <v>3</v>
@@ -83064,10 +83064,10 @@
         </is>
       </c>
       <c r="C4591" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4591" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4592">
@@ -83082,7 +83082,7 @@
         </is>
       </c>
       <c r="C4592" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4592" t="n">
         <v>4</v>
@@ -83100,10 +83100,10 @@
         </is>
       </c>
       <c r="C4593" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4593" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4594">
@@ -83118,7 +83118,7 @@
         </is>
       </c>
       <c r="C4594" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4594" t="n">
         <v>3</v>
@@ -83127,16 +83127,16 @@
     <row r="4595">
       <c r="A4595" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4595" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4595" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4595" t="n">
         <v>3</v>
@@ -83154,9 +83154,27 @@
         </is>
       </c>
       <c r="C4596" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4596" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4597">
+      <c r="A4597" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4597" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4597" t="n">
         <v>7</v>
       </c>
-      <c r="D4596" t="n">
+      <c r="D4597" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto push: 2026-09-05 04:22 UTC
</commit_message>
<xml_diff>
--- a/excel/apple3.xlsx
+++ b/excel/apple3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4644"/>
+  <dimension ref="A1:D4645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83271,19 +83271,19 @@
     <row r="4603">
       <c r="A4603" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="B4603" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4603" t="n">
         <v>13</v>
       </c>
       <c r="D4603" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4604">
@@ -83298,7 +83298,7 @@
         </is>
       </c>
       <c r="C4604" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4604" t="n">
         <v>3</v>
@@ -83316,7 +83316,7 @@
         </is>
       </c>
       <c r="C4605" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4605" t="n">
         <v>3</v>
@@ -83334,7 +83334,7 @@
         </is>
       </c>
       <c r="C4606" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4606" t="n">
         <v>3</v>
@@ -83343,16 +83343,16 @@
     <row r="4607">
       <c r="A4607" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B4607" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C4607" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D4607" t="n">
         <v>3</v>
@@ -83370,7 +83370,7 @@
         </is>
       </c>
       <c r="C4608" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4608" t="n">
         <v>3</v>
@@ -83388,7 +83388,7 @@
         </is>
       </c>
       <c r="C4609" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4609" t="n">
         <v>3</v>
@@ -83406,7 +83406,7 @@
         </is>
       </c>
       <c r="C4610" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4610" t="n">
         <v>3</v>
@@ -83424,7 +83424,7 @@
         </is>
       </c>
       <c r="C4611" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4611" t="n">
         <v>3</v>
@@ -83442,7 +83442,7 @@
         </is>
       </c>
       <c r="C4612" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D4612" t="n">
         <v>3</v>
@@ -83451,16 +83451,16 @@
     <row r="4613">
       <c r="A4613" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B4613" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C4613" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4613" t="n">
         <v>3</v>
@@ -83478,7 +83478,7 @@
         </is>
       </c>
       <c r="C4614" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D4614" t="n">
         <v>3</v>
@@ -83496,7 +83496,7 @@
         </is>
       </c>
       <c r="C4615" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4615" t="n">
         <v>3</v>
@@ -83514,7 +83514,7 @@
         </is>
       </c>
       <c r="C4616" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4616" t="n">
         <v>3</v>
@@ -83532,7 +83532,7 @@
         </is>
       </c>
       <c r="C4617" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D4617" t="n">
         <v>3</v>
@@ -83550,7 +83550,7 @@
         </is>
       </c>
       <c r="C4618" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D4618" t="n">
         <v>3</v>
@@ -83559,16 +83559,16 @@
     <row r="4619">
       <c r="A4619" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B4619" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C4619" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4619" t="n">
         <v>3</v>
@@ -83586,7 +83586,7 @@
         </is>
       </c>
       <c r="C4620" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D4620" t="n">
         <v>3</v>
@@ -83604,7 +83604,7 @@
         </is>
       </c>
       <c r="C4621" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D4621" t="n">
         <v>3</v>
@@ -83622,7 +83622,7 @@
         </is>
       </c>
       <c r="C4622" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4622" t="n">
         <v>3</v>
@@ -83640,7 +83640,7 @@
         </is>
       </c>
       <c r="C4623" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4623" t="n">
         <v>3</v>
@@ -83649,16 +83649,16 @@
     <row r="4624">
       <c r="A4624" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B4624" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C4624" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D4624" t="n">
         <v>3</v>
@@ -83676,7 +83676,7 @@
         </is>
       </c>
       <c r="C4625" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4625" t="n">
         <v>3</v>
@@ -83694,7 +83694,7 @@
         </is>
       </c>
       <c r="C4626" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4626" t="n">
         <v>3</v>
@@ -83712,10 +83712,10 @@
         </is>
       </c>
       <c r="C4627" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4627" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4628">
@@ -83730,7 +83730,7 @@
         </is>
       </c>
       <c r="C4628" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4628" t="n">
         <v>2</v>
@@ -83748,7 +83748,7 @@
         </is>
       </c>
       <c r="C4629" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4629" t="n">
         <v>2</v>
@@ -83766,7 +83766,7 @@
         </is>
       </c>
       <c r="C4630" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4630" t="n">
         <v>2</v>
@@ -83775,16 +83775,16 @@
     <row r="4631">
       <c r="A4631" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B4631" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C4631" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4631" t="n">
         <v>2</v>
@@ -83802,10 +83802,10 @@
         </is>
       </c>
       <c r="C4632" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4632" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4633">
@@ -83820,7 +83820,7 @@
         </is>
       </c>
       <c r="C4633" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4633" t="n">
         <v>3</v>
@@ -83838,7 +83838,7 @@
         </is>
       </c>
       <c r="C4634" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4634" t="n">
         <v>3</v>
@@ -83856,7 +83856,7 @@
         </is>
       </c>
       <c r="C4635" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D4635" t="n">
         <v>3</v>
@@ -83874,7 +83874,7 @@
         </is>
       </c>
       <c r="C4636" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4636" t="n">
         <v>3</v>
@@ -83892,7 +83892,7 @@
         </is>
       </c>
       <c r="C4637" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4637" t="n">
         <v>3</v>
@@ -83901,16 +83901,16 @@
     <row r="4638">
       <c r="A4638" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B4638" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4638" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D4638" t="n">
         <v>3</v>
@@ -83928,10 +83928,10 @@
         </is>
       </c>
       <c r="C4639" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4639" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4640">
@@ -83946,7 +83946,7 @@
         </is>
       </c>
       <c r="C4640" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4640" t="n">
         <v>4</v>
@@ -83964,10 +83964,10 @@
         </is>
       </c>
       <c r="C4641" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4641" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4642">
@@ -83982,7 +83982,7 @@
         </is>
       </c>
       <c r="C4642" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4642" t="n">
         <v>3</v>
@@ -83991,16 +83991,16 @@
     <row r="4643">
       <c r="A4643" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B4643" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C4643" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D4643" t="n">
         <v>3</v>
@@ -84018,9 +84018,27 @@
         </is>
       </c>
       <c r="C4644" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4644" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4645">
+      <c r="A4645" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B4645" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C4645" t="n">
         <v>7</v>
       </c>
-      <c r="D4644" t="n">
+      <c r="D4645" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>